<commit_message>
Final numerical reconciliation and package submission for ETCCDI Chiang Mai project
Co-authored-by: surasit3173 <247266065+surasit3173@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ETCCDI_ChiangMai/audit/INDEPENDENT_VERIFICATION.xlsx
+++ b/ETCCDI_ChiangMai/audit/INDEPENDENT_VERIFICATION.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -807,17 +807,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Primary Trend (Ordinary_MK) — PRCPTOT</t>
+          <t>Primary Test (Ordinary_MK) — PRCPTOT</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Tau=-0.0847, Slope=-1.5311, P=0.346353</t>
+          <t>Tau=-0.0847, Slope=-1.5311, P=0.346353, Z=-0.9417, S=-145.0, VarS=23383.67</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Tau=-0.0847, Slope=-1.5311, P=0.346353</t>
+          <t>Tau=-0.0847, Slope=-1.5311, P=0.346353, Z=-0.9417, S=-145.0, VarS=23383.67</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -835,17 +835,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Primary Trend (Ordinary_MK) — SDII</t>
+          <t>Primary Test (Ordinary_MK) — SDII</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Tau=-0.0935, Slope=-0.0104, P=0.298412</t>
+          <t>Tau=-0.0935, Slope=-0.0104, P=0.298412, Z=-1.0398, S=-160.0, VarS=23380.67</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Tau=-0.0935, Slope=-0.0104, P=0.298412</t>
+          <t>Tau=-0.0935, Slope=-0.0104, P=0.298412, Z=-1.0398, S=-160.0, VarS=23380.67</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -863,17 +863,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Primary Trend (Ordinary_MK) — Rx1day</t>
+          <t>Primary Test (Ordinary_MK) — Rx1day</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Tau=0.0643, Slope=0.1632, P=0.475958</t>
+          <t>Tau=0.0643, Slope=0.1632, P=0.475958, Z=0.7128, S=110.0, VarS=23382.67</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Tau=0.0643, Slope=0.1632, P=0.475958</t>
+          <t>Tau=0.0643, Slope=0.1632, P=0.475958, Z=0.7128, S=110.0, VarS=23382.67</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -891,17 +891,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Primary Trend (Ordinary_MK) — Rx5day</t>
+          <t>Primary Test (Ordinary_MK) — Rx5day</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Tau=-0.0105, Slope=-0.0435, P=0.911479</t>
+          <t>Tau=-0.0105, Slope=-0.0435, P=0.911479, Z=-0.1112, S=-18.0, VarS=23382.67</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Tau=-0.0105, Slope=-0.0435, P=0.911479</t>
+          <t>Tau=-0.0105, Slope=-0.0435, P=0.911479, Z=-0.1112, S=-18.0, VarS=23382.67</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -919,17 +919,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Primary Trend (Ordinary_MK) — CDD</t>
+          <t>Primary Test (Ordinary_MK) — CDD</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Tau=0.0503, Slope=0.1212, P=0.578214</t>
+          <t>Tau=0.0503, Slope=0.1212, P=0.578214, Z=0.5560, S=86.0, VarS=23372.00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Tau=0.0503, Slope=0.1212, P=0.578214</t>
+          <t>Tau=0.0503, Slope=0.1212, P=0.578214, Z=0.5560, S=86.0, VarS=23372.00</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -947,17 +947,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Primary Trend (Ordinary_MK) — CWD</t>
+          <t>Primary Test (Ordinary_MK) — CWD</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Tau=-0.0526, Slope=0.0000, P=0.556118</t>
+          <t>Tau=-0.0526, Slope=0.0000, P=0.556118, Z=-0.5886, S=-90.0, VarS=22862.00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Tau=-0.0526, Slope=-0.0000, P=0.556118</t>
+          <t>Tau=-0.0526, Slope=-0.0000, P=0.556118, Z=-0.5886, S=-90.0, VarS=22862.00</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -975,17 +975,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Primary Trend (Ordinary_MK) — R10mm</t>
+          <t>Primary Test (Ordinary_MK) — R10mm</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Tau=-0.0240, Slope=0.0000, P=0.793285</t>
+          <t>Tau=-0.0240, Slope=0.0000, P=0.793285, Z=-0.2620, S=-41.0, VarS=23300.33</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Tau=-0.0240, Slope=-0.0000, P=0.793285</t>
+          <t>Tau=-0.0240, Slope=-0.0000, P=0.793285, Z=-0.2620, S=-41.0, VarS=23300.33</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1003,17 +1003,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Primary Trend (Ordinary_MK) — R20mm</t>
+          <t>Primary Test (Ordinary_MK) — R20mm</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Tau=-0.0959, Slope=-0.0370, P=0.284601</t>
+          <t>Tau=-0.0959, Slope=-0.0370, P=0.284601, Z=-1.0700, S=-164.0, VarS=23204.67</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Tau=-0.0959, Slope=-0.0370, P=0.284601</t>
+          <t>Tau=-0.0959, Slope=-0.0370, P=0.284601, Z=-1.0700, S=-164.0, VarS=23204.67</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1031,17 +1031,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Primary Trend (Hamed_Rao_modified_MK) — R50mm</t>
+          <t>Primary Test (Hamed_Rao_modified_MK) — R50mm</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Tau=-0.0579, Slope=0.0000, P=0.451230</t>
+          <t>Tau=-0.0579, Slope=0.0000, P=0.451230, Z=-0.7534, S=-99.0, VarS=16921.51</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Tau=-0.0579, Slope=-0.0000, P=0.451230</t>
+          <t>Tau=-0.0579, Slope=-0.0000, P=0.451230, Z=-0.7534, S=-99.0, VarS=16921.51</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1059,17 +1059,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Primary Trend (Ordinary_MK) — R95p</t>
+          <t>Primary Test (Ordinary_MK) — R95p</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Tau=-0.0678, Slope=-0.7786, P=0.452017</t>
+          <t>Tau=-0.0678, Slope=-0.7786, P=0.452017, Z=-0.7521, S=-116.0, VarS=23382.67</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Tau=-0.0678, Slope=-0.7786, P=0.452017</t>
+          <t>Tau=-0.0678, Slope=-0.7786, P=0.452017, Z=-0.7521, S=-116.0, VarS=23382.67</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1087,17 +1087,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Primary Trend (Hamed_Rao_modified_MK) — R99p</t>
+          <t>Primary Test (Hamed_Rao_modified_MK) — R99p</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Tau=0.0222, Slope=0.0000, P=0.532865</t>
+          <t>Tau=0.0222, Slope=0.0000, P=0.532865, Z=0.6236, S=38.0, VarS=3519.96</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Tau=0.0222, Slope=-0.0000, P=0.532865</t>
+          <t>Tau=0.0222, Slope=-0.0000, P=0.532865, Z=0.6236, S=38.0, VarS=3519.96</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1107,6 +1107,34 @@
         <v>0.001</v>
       </c>
       <c r="F25" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>BH-FDR Adjusted P-Values (All 11 Indices)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Min FDR P = 0.706706</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Min FDR P = 0.706706</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="F26" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>

</xml_diff>